<commit_message>
Audit global : abonnement sur mesure, sceau sans COFRAC, BMC aligné, BP avec feuille de route et hypothèses, pitch mis à jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013D7uRxLFz2dHeA6eheZQbo
</commit_message>
<xml_diff>
--- a/livrable/Business_Plan_PCE.xlsx
+++ b/livrable/Business_Plan_PCE.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feuille 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypothèses" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12,10 +13,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="# ##0"/>
+    <numFmt numFmtId="166" formatCode="# ##0 €"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="8">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -38,8 +41,25 @@
       <color rgb="FF000000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00023481"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00023481"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +78,11 @@
         <bgColor rgb="FFD8EAF9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00023481"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -65,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -111,6 +136,39 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -499,14 +557,14 @@
           <t>TAILLE DU MARCHE</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="16" t="n">
         <v>250000</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="17">
         <f>IF(OR(B5="",C4=""),"",B5*(1+C4))</f>
         <v/>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="17">
         <f>IF(OR(C5="",D4=""),"",C5*(1+D4))</f>
         <v/>
       </c>
@@ -533,14 +591,14 @@
           <t>QUANTITES VENDUES</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="16" t="n">
         <v>500</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="17">
         <f>IF(OR(C5="",C6=""),"",C5*C6)</f>
         <v/>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="17">
         <f>IF(OR(D5="",D6=""),"",D5*D6)</f>
         <v/>
       </c>
@@ -551,13 +609,13 @@
           <t>PRIX DE VENTE UNITAIRE</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="18" t="n">
         <v>137</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="19" t="n">
         <v>137</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="19" t="n">
         <v>137</v>
       </c>
     </row>
@@ -567,15 +625,15 @@
           <t>CHIFFRE D’AFFAIRES HORS TAXES</t>
         </is>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="20">
         <f>IF(OR(B7="",B8=""),"",B7*B8)</f>
         <v/>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="20">
         <f>IF(OR(C7="",C8=""),"",C7*C8)</f>
         <v/>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="20">
         <f>IF(OR(D7="",D8=""),"",D7*D8)</f>
         <v/>
       </c>
@@ -596,13 +654,13 @@
           <t>ACHATS MARCHANDISES</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="10" t="n">
+      <c r="B11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -612,13 +670,13 @@
           <t>ACHATS MATIERES PREMIERES</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="10" t="n">
+      <c r="B12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -628,13 +686,13 @@
           <t>LOYERS</t>
         </is>
       </c>
-      <c r="B13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="10" t="n">
+      <c r="B13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -644,13 +702,13 @@
           <t>PUBLICITE</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="19" t="n">
         <v>15000</v>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="19" t="n">
         <v>25000</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="19" t="n">
         <v>35000</v>
       </c>
     </row>
@@ -660,13 +718,13 @@
           <t>FRAIS DEPLACEMENT</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="19" t="n">
         <v>3000</v>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="19" t="n">
         <v>4000</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="19" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -676,13 +734,13 @@
           <t>TELEPHONIE</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="19" t="n">
         <v>1200</v>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C16" s="19" t="n">
         <v>1500</v>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D16" s="19" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -692,13 +750,13 @@
           <t>MAINTENANCE MATERIELS</t>
         </is>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="19" t="n">
         <v>2400</v>
       </c>
-      <c r="C17" s="10" t="n">
+      <c r="C17" s="19" t="n">
         <v>3600</v>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D17" s="19" t="n">
         <v>4800</v>
       </c>
     </row>
@@ -708,14 +766,14 @@
           <t>SOUS-TRAITANCE</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C18" s="10" t="n">
-        <v>50250</v>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>102225</v>
+      <c r="B18" s="19" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>65250</v>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>110225</v>
       </c>
     </row>
     <row r="19">
@@ -724,13 +782,13 @@
           <t>IMPOTS ET TAXES</t>
         </is>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="19" t="n">
         <v>500</v>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="19" t="n">
         <v>1500</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="19" t="n">
         <v>3000</v>
       </c>
     </row>
@@ -740,13 +798,13 @@
           <t>SALAIRES ET TRAITEMENTS</t>
         </is>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="19" t="n">
         <v>30000</v>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="19" t="n">
         <v>50000</v>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="D20" s="19" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -756,13 +814,13 @@
           <t>CHARGES SOCIALES</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="19" t="n">
         <v>12600</v>
       </c>
-      <c r="C21" s="10" t="n">
+      <c r="C21" s="19" t="n">
         <v>21000</v>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="19" t="n">
         <v>50400</v>
       </c>
     </row>
@@ -772,15 +830,15 @@
           <t>TOTAL DES CHARGES D’EXPLOITATION</t>
         </is>
       </c>
-      <c r="B22" s="9">
+      <c r="B22" s="20">
         <f>IF(COUNT(B11:B21)=0,"",SUM(B11:B21))</f>
         <v/>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="20">
         <f>IF(COUNT(C11:C21)=0,"",SUM(C11:C21))</f>
         <v/>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="20">
         <f>IF(COUNT(D11:D21)=0,"",SUM(D11:D21))</f>
         <v/>
       </c>
@@ -791,15 +849,15 @@
           <t>EXCEDENT BRUT EXPLOITATION (EBE ou EBITA)</t>
         </is>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="20">
         <f>IF(OR(B9="",B22=""),"",B9-B22)</f>
         <v/>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="20">
         <f>IF(OR(C9="",C22=""),"",C9-C22)</f>
         <v/>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="20">
         <f>IF(OR(D9="",D22=""),"",D9-D22)</f>
         <v/>
       </c>
@@ -852,15 +910,15 @@
           <t>EBE</t>
         </is>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="20">
         <f>IF(B23="","",B23)</f>
         <v/>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="20">
         <f>IF(C23="","",C23)</f>
         <v/>
       </c>
-      <c r="D28" s="9">
+      <c r="D28" s="20">
         <f>IF(D23="","",D23)</f>
         <v/>
       </c>
@@ -871,29 +929,29 @@
           <t>APPORT EN CAPITAL</t>
         </is>
       </c>
-      <c r="B29" s="10" t="n">
+      <c r="B29" s="19" t="n">
         <v>10000</v>
       </c>
-      <c r="C29" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="10" t="n">
+      <c r="C29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>APPORT EN COOMPTE COURANT ASSOCIES</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="10" t="n">
+          <t>APPORT EN COMPTE COURANT ASSOCIES</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -903,13 +961,13 @@
           <t>SUBVENTION INVESTISSEMENT</t>
         </is>
       </c>
-      <c r="B31" s="10" t="n">
+      <c r="B31" s="19" t="n">
         <v>15000</v>
       </c>
-      <c r="C31" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="10" t="n">
+      <c r="C31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -919,13 +977,13 @@
           <t>EMPRUNT BANCAIRE</t>
         </is>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="19" t="n">
         <v>50000</v>
       </c>
-      <c r="C32" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="10" t="n">
+      <c r="C32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -935,15 +993,15 @@
           <t>TOTAL DES RESSOURCES (1)</t>
         </is>
       </c>
-      <c r="B33" s="9">
+      <c r="B33" s="20">
         <f>IF(B28="","",SUM(B28:B32))</f>
         <v/>
       </c>
-      <c r="C33" s="9">
+      <c r="C33" s="20">
         <f>IF(C28="","",SUM(C28:C32))</f>
         <v/>
       </c>
-      <c r="D33" s="9">
+      <c r="D33" s="20">
         <f>IF(D28="","",SUM(D28:D32))</f>
         <v/>
       </c>
@@ -964,13 +1022,13 @@
           <t>INVESTISSEMENTS INCORPORELS</t>
         </is>
       </c>
-      <c r="B35" s="10" t="n">
+      <c r="B35" s="19" t="n">
         <v>30000</v>
       </c>
-      <c r="C35" s="10" t="n">
+      <c r="C35" s="19" t="n">
         <v>5000</v>
       </c>
-      <c r="D35" s="10" t="n">
+      <c r="D35" s="19" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -980,13 +1038,13 @@
           <t>INVESTISSEMENTS CORPORELS</t>
         </is>
       </c>
-      <c r="B36" s="10" t="n">
+      <c r="B36" s="19" t="n">
         <v>4000</v>
       </c>
-      <c r="C36" s="10" t="n">
+      <c r="C36" s="19" t="n">
         <v>1000</v>
       </c>
-      <c r="D36" s="10" t="n">
+      <c r="D36" s="19" t="n">
         <v>1000</v>
       </c>
     </row>
@@ -996,13 +1054,13 @@
           <t>INVESTISSEMENTS FINANCIERS</t>
         </is>
       </c>
-      <c r="B37" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C37" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="10" t="n">
+      <c r="B37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1012,13 +1070,13 @@
           <t>AUGMENTATION DU BESOIN EN FONDS DE ROULEMENT</t>
         </is>
       </c>
-      <c r="B38" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C38" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="10" t="n">
+      <c r="B38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1028,13 +1086,13 @@
           <t>REMBOURSEMENT EMPRUNT BANCAIRE</t>
         </is>
       </c>
-      <c r="B39" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C39" s="10" t="n">
+      <c r="B39" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="19" t="n">
         <v>8000</v>
       </c>
-      <c r="D39" s="10" t="n">
+      <c r="D39" s="19" t="n">
         <v>8000</v>
       </c>
     </row>
@@ -1044,15 +1102,15 @@
           <t>TOTAL DES EMPLOIS (2)</t>
         </is>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="20">
         <f>IF(COUNT(B35:B39)=0,"",SUM(B35:B39))</f>
         <v/>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="20">
         <f>IF(COUNT(C35:C39)=0,"",SUM(C35:C39))</f>
         <v/>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="20">
         <f>IF(COUNT(D35:D39)=0,"",SUM(D35:D39))</f>
         <v/>
       </c>
@@ -1063,15 +1121,15 @@
           <t>VARIATION DE LA TRESORERIE = (1) – (2)</t>
         </is>
       </c>
-      <c r="B41" s="9">
+      <c r="B41" s="20">
         <f>IF(OR(B33="",B40=""),"",B33-B40)</f>
         <v/>
       </c>
-      <c r="C41" s="9">
+      <c r="C41" s="20">
         <f>IF(OR(C33="",C40=""),"",C33-C40)</f>
         <v/>
       </c>
-      <c r="D41" s="9">
+      <c r="D41" s="20">
         <f>IF(OR(D33="",D40=""),"",D33-D40)</f>
         <v/>
       </c>
@@ -1082,14 +1140,14 @@
           <t>TRESORERIE INITIALE</t>
         </is>
       </c>
-      <c r="B42" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" s="9">
+      <c r="B42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="20">
         <f>IF(B43="","",B43)</f>
         <v/>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="20">
         <f>IF(C43="","",C43)</f>
         <v/>
       </c>
@@ -1100,15 +1158,15 @@
           <t>TRESORERIE FINALE</t>
         </is>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="20">
         <f>IF(OR(B42="",B41=""),"",B42+B41)</f>
         <v/>
       </c>
-      <c r="C43" s="9">
+      <c r="C43" s="20">
         <f>IF(OR(C42="",C41=""),"",C42+C41)</f>
         <v/>
       </c>
-      <c r="D43" s="9">
+      <c r="D43" s="20">
         <f>IF(OR(D42="",D41=""),"",D42+D41)</f>
         <v/>
       </c>
@@ -1117,4 +1175,266 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" style="13" min="1" max="1"/>
+    <col width="110" customWidth="1" style="13" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>HYPOTHÈSES DU BUSINESS PLAN PCE</t>
+        </is>
+      </c>
+      <c r="B1" s="22" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>Toutes les valeurs sont des hypothèses de travail, à valider. Montants hors taxes.</t>
+        </is>
+      </c>
+      <c r="B2" s="22" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="22" t="n"/>
+      <c r="B3" s="22" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Marché et clients</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>Marché visé</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>250 000 créatifs (indépendants, studios, agences) en France. Chiffre non sourcé, à vérifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Croissance du marché</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>5 % par an.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Part de marché</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>0,2 % en année 1 (500 clients), 0,6 % en année 2 (1 575), 1,2 % en année 3 (3 308).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>Phase pilote</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>100 freelances pilotes certifiés en début d'année 1, puis 500 clients payants en fin d'année 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="n"/>
+      <c r="B9" s="22" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Prix</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>Revenu moyen par client</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>137 € HT par an : abonnement sur mesure et certifications à l'unité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>Abonnement sur mesure</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>Indépendant à partir de 9 € HT/mois (6 créations/an incluses). Studio (2 à 10 personnes) à partir de 29 € (24 incluses). Agence (11 à 50) à partir de 79 € (60 incluses). Grand compte sur devis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>Variables du tarif</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>+0,50 € HT/mois par création au-delà du volume inclus. Processus moyen (10 à 40 h) +3 €, long (plus de 40 h) +8 €. Étude du dossier : incluse (indépendant), 49 € (studio), 149 € (agence), une seule fois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>Certification à l'unité</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>Selon l'œuvre : photographie 25 €, illustration 29 €, tatouage 39 €, identité visuelle 49 €, campagne de marque 149 €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>Vérification</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Gratuite pour l'acheteur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="n"/>
+      <c r="B16" s="22" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Charges</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>Sous-traitance</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Jury de vérification à 30 € par dossier, plus 5 000 € de juridique en année 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>Feuille de route (dans la sous-traitance)</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>Année 1 : co-construction du référentiel avec l'AFNOR, 5 000 €. Année 2 : audits COFRAC (documentaire, sur site, accompagnement), 15 000 €. Année 3 : audit de surveillance COFRAC, 8 000 €. Montants estimés, non vérifiés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Publicité</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>15 000 €, 25 000 €, 35 000 €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Salaires</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>30 000 €, 50 000 €, 120 000 €. Charges sociales à 42 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="n"/>
+      <c r="B22" s="22" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>Financement</t>
+        </is>
+      </c>
+      <c r="B23" s="25" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>Apports</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>10 000 € de capital (4 associés), 15 000 € de subvention, 50 000 € d'emprunt remboursé 8 000 € par an à partir de l'année 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>Investissements</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>Plateforme et marque : 30 000 € en année 1, puis 5 000 € par an. Matériel : 4 000 € en année 1, puis 1 000 € par an.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>